<commit_message>
Update eMed mapping with correct hierarchy level for doseQuantity element
</commit_message>
<xml_diff>
--- a/python-maps/documentation/CDA2FHIR_elga_eMed_groups.xlsx
+++ b/python-maps/documentation/CDA2FHIR_elga_eMed_groups.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maximilian/Documents/BlackTusk/Bundesrechenzentrum/CDA2FHIR/CDA2FHIR/python-maps/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6903998-BB95-6D41-A79A-718C304FC4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{374371A5-9F37-8043-9243-064C66F7F4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1293" uniqueCount="475">
   <si>
     <t xml:space="preserve">Status
 </t>
@@ -1371,12 +1371,6 @@
     <t>sA/effectiveTime/period/@unit</t>
   </si>
   <si>
-    <t>sA/effectiveTime/doseQuantity/@value</t>
-  </si>
-  <si>
-    <t>sA/effectiveTime/doseQuantity/@unit</t>
-  </si>
-  <si>
     <t>sA/entryRelationship/@typeCode='COMP'</t>
   </si>
   <si>
@@ -1636,9 +1630,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -2123,167 +2124,167 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="164">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2292,252 +2293,253 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3125,7 +3127,7 @@
       <c r="K5" s="7"/>
       <c r="L5" s="20"/>
       <c r="M5" s="7" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="N5" s="7"/>
     </row>
@@ -3569,7 +3571,7 @@
         <v>36</v>
       </c>
       <c r="D14" s="84" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="E14" s="82"/>
       <c r="F14" s="87"/>
@@ -3592,7 +3594,7 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="154" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B15" s="154"/>
       <c r="C15" s="154"/>
@@ -3619,7 +3621,7 @@
         <v>36</v>
       </c>
       <c r="D16" s="81" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="E16" s="82"/>
       <c r="F16" s="87"/>
@@ -3643,7 +3645,7 @@
         <v>36</v>
       </c>
       <c r="D17" s="97" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E17" s="82"/>
       <c r="F17" s="87"/>
@@ -3667,7 +3669,7 @@
         <v>36</v>
       </c>
       <c r="D18" s="97" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="E18" s="82"/>
       <c r="F18" s="87"/>
@@ -3691,7 +3693,7 @@
         <v>36</v>
       </c>
       <c r="D19" s="81" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="E19" s="82"/>
       <c r="F19" s="87"/>
@@ -3715,7 +3717,7 @@
         <v>36</v>
       </c>
       <c r="D20" s="81" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="E20" s="82"/>
       <c r="F20" s="87"/>
@@ -3739,7 +3741,7 @@
         <v>36</v>
       </c>
       <c r="D21" s="97" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E21" s="82"/>
       <c r="F21" s="87"/>
@@ -3763,7 +3765,7 @@
         <v>36</v>
       </c>
       <c r="D22" s="81" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E22" s="82"/>
       <c r="F22" s="87"/>
@@ -3787,7 +3789,7 @@
         <v>36</v>
       </c>
       <c r="D23" s="81" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E23" s="82"/>
       <c r="F23" s="87"/>
@@ -3817,14 +3819,14 @@
         <v>36</v>
       </c>
       <c r="D24" s="81" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="E24" s="82"/>
       <c r="F24" s="87"/>
       <c r="G24" s="87"/>
       <c r="H24" s="82"/>
       <c r="I24" s="81" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="J24" s="83" t="s">
         <v>240</v>
@@ -3845,7 +3847,7 @@
         <v>36</v>
       </c>
       <c r="D25" s="81" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="E25" s="82"/>
       <c r="F25" s="87"/>
@@ -3875,7 +3877,7 @@
         <v>36</v>
       </c>
       <c r="D26" s="81" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="E26" s="82"/>
       <c r="F26" s="87"/>
@@ -3903,7 +3905,7 @@
         <v>36</v>
       </c>
       <c r="D27" s="81" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="E27" s="82"/>
       <c r="F27" s="93" t="s">
@@ -3933,7 +3935,7 @@
         <v>36</v>
       </c>
       <c r="D28" s="81" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E28" s="82"/>
       <c r="F28" s="87"/>
@@ -3957,7 +3959,7 @@
         <v>36</v>
       </c>
       <c r="D29" s="81" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E29" s="82"/>
       <c r="F29" s="87"/>
@@ -3981,7 +3983,7 @@
         <v>36</v>
       </c>
       <c r="D30" s="81" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="E30" s="82"/>
       <c r="F30" s="87"/>
@@ -4009,7 +4011,7 @@
         <v>36</v>
       </c>
       <c r="D31" s="81" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E31" s="82"/>
       <c r="F31" s="87"/>
@@ -4033,7 +4035,7 @@
         <v>36</v>
       </c>
       <c r="D32" s="81" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="E32" s="82"/>
       <c r="F32" s="87"/>
@@ -4057,7 +4059,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="81" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E33" s="82"/>
       <c r="F33" s="87"/>
@@ -4081,7 +4083,7 @@
         <v>36</v>
       </c>
       <c r="D34" s="81" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E34" s="82"/>
       <c r="F34" s="87"/>
@@ -4111,7 +4113,7 @@
         <v>36</v>
       </c>
       <c r="D35" s="81" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E35" s="82"/>
       <c r="F35" s="87"/>
@@ -4141,7 +4143,7 @@
         <v>36</v>
       </c>
       <c r="D36" s="81" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E36" s="82"/>
       <c r="F36" s="87"/>
@@ -4169,7 +4171,7 @@
         <v>36</v>
       </c>
       <c r="D37" s="81" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="E37" s="82"/>
       <c r="F37" s="87" t="s">
@@ -4201,7 +4203,7 @@
         <v>36</v>
       </c>
       <c r="D38" s="81" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="E38" s="82"/>
       <c r="F38" s="87"/>
@@ -4222,7 +4224,7 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A39" s="151" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B39" s="152"/>
       <c r="C39" s="152"/>
@@ -4246,17 +4248,17 @@
       </c>
       <c r="B40" s="94"/>
       <c r="C40" s="83" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D40" s="81" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="E40" s="82"/>
       <c r="F40" s="87"/>
       <c r="G40" s="87"/>
       <c r="H40" s="82"/>
       <c r="I40" s="85" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="J40" s="83"/>
       <c r="K40" s="83"/>
@@ -4272,17 +4274,17 @@
       </c>
       <c r="B41" s="94"/>
       <c r="C41" s="83" t="s">
+        <v>466</v>
+      </c>
+      <c r="D41" s="81" t="s">
         <v>468</v>
-      </c>
-      <c r="D41" s="81" t="s">
-        <v>470</v>
       </c>
       <c r="E41" s="82"/>
       <c r="F41" s="87"/>
       <c r="G41" s="87"/>
       <c r="H41" s="82"/>
       <c r="I41" s="85" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="J41" s="83" t="s">
         <v>240</v>
@@ -4444,7 +4446,7 @@
       <c r="K47" s="83"/>
       <c r="L47" s="82"/>
       <c r="M47" s="81" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="N47" s="82"/>
       <c r="O47" s="82"/>
@@ -4470,7 +4472,7 @@
       <c r="K48" s="83"/>
       <c r="L48" s="82"/>
       <c r="M48" s="85" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="N48" s="82"/>
       <c r="O48" s="82"/>
@@ -4646,7 +4648,7 @@
       <c r="K55" s="83"/>
       <c r="L55" s="82"/>
       <c r="M55" s="81" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="N55" s="82"/>
       <c r="O55" s="82"/>
@@ -4672,7 +4674,7 @@
       <c r="K56" s="83"/>
       <c r="L56" s="82"/>
       <c r="M56" s="85" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="N56" s="82"/>
       <c r="O56" s="82"/>
@@ -4984,7 +4986,7 @@
       <c r="G69" s="87"/>
       <c r="H69" s="82"/>
       <c r="I69" s="86" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="J69" s="94"/>
       <c r="K69" s="83"/>
@@ -5434,7 +5436,7 @@
       <c r="G87" s="87"/>
       <c r="H87" s="82"/>
       <c r="I87" s="86" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="J87" s="94"/>
       <c r="K87" s="83"/>
@@ -5857,7 +5859,7 @@
       <c r="K104" s="83"/>
       <c r="L104" s="82"/>
       <c r="M104" s="81" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="N104" s="82"/>
       <c r="O104" s="82"/>
@@ -5887,7 +5889,7 @@
       <c r="K105" s="83"/>
       <c r="L105" s="82"/>
       <c r="M105" s="81" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="N105" s="82"/>
       <c r="O105" s="82"/>
@@ -8271,7 +8273,7 @@
         <v>36</v>
       </c>
       <c r="D199" s="123" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="E199" s="82"/>
       <c r="F199" s="87"/>
@@ -8299,7 +8301,7 @@
         <v>257</v>
       </c>
       <c r="D200" s="123" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="E200" s="82"/>
       <c r="F200" s="93" t="s">
@@ -8331,7 +8333,7 @@
         <v>36</v>
       </c>
       <c r="D201" s="123" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E201" s="82"/>
       <c r="F201" s="87"/>
@@ -8357,7 +8359,7 @@
         <v>36</v>
       </c>
       <c r="D202" s="123" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E202" s="82"/>
       <c r="F202" s="87"/>
@@ -8381,7 +8383,7 @@
         <v>36</v>
       </c>
       <c r="D203" s="123" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E203" s="82"/>
       <c r="F203" s="87"/>
@@ -8409,7 +8411,7 @@
         <v>36</v>
       </c>
       <c r="D204" s="123" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E204" s="82"/>
       <c r="F204" s="87"/>
@@ -8433,7 +8435,7 @@
         <v>36</v>
       </c>
       <c r="D205" s="123" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E205" s="82"/>
       <c r="F205" s="87"/>
@@ -8457,7 +8459,7 @@
         <v>36</v>
       </c>
       <c r="D206" s="123" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E206" s="82"/>
       <c r="F206" s="87" t="s">
@@ -8495,7 +8497,7 @@
         <v>36</v>
       </c>
       <c r="D207" s="123" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="E207" s="82"/>
       <c r="F207" s="87"/>
@@ -8523,7 +8525,7 @@
         <v>36</v>
       </c>
       <c r="D208" s="123" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="E208" s="82"/>
       <c r="F208" s="87"/>
@@ -8551,7 +8553,7 @@
         <v>36</v>
       </c>
       <c r="D209" s="123" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="E209" s="82"/>
       <c r="F209" s="87"/>
@@ -8579,7 +8581,7 @@
         <v>257</v>
       </c>
       <c r="D210" s="123" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E210" s="82"/>
       <c r="F210" s="93" t="s">
@@ -8663,7 +8665,7 @@
         <v>281</v>
       </c>
       <c r="D213" s="124" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="E213" s="82"/>
       <c r="F213" s="87"/>
@@ -8689,7 +8691,7 @@
         <v>36</v>
       </c>
       <c r="D214" s="125" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E214" s="82"/>
       <c r="F214" s="87"/>
@@ -8717,7 +8719,7 @@
         <v>36</v>
       </c>
       <c r="D215" s="126" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="E215" s="82"/>
       <c r="F215" s="87"/>
@@ -8745,7 +8747,7 @@
         <v>36</v>
       </c>
       <c r="D216" s="126" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E216" s="82"/>
       <c r="F216" s="87" t="s">
@@ -8774,8 +8776,8 @@
       <c r="C217" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="D217" s="123" t="s">
-        <v>391</v>
+      <c r="D217" s="164" t="s">
+        <v>432</v>
       </c>
       <c r="E217" s="82"/>
       <c r="F217" s="87"/>
@@ -8802,8 +8804,8 @@
       <c r="C218" s="115" t="s">
         <v>257</v>
       </c>
-      <c r="D218" s="123" t="s">
-        <v>392</v>
+      <c r="D218" s="164" t="s">
+        <v>433</v>
       </c>
       <c r="E218" s="82"/>
       <c r="F218" s="93" t="s">
@@ -8835,7 +8837,7 @@
         <v>36</v>
       </c>
       <c r="D219" s="123" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E219" s="82"/>
       <c r="F219" s="87"/>
@@ -8861,7 +8863,7 @@
         <v>36</v>
       </c>
       <c r="D220" s="123" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="E220" s="82"/>
       <c r="F220" s="87"/>
@@ -8885,7 +8887,7 @@
         <v>36</v>
       </c>
       <c r="D221" s="123" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E221" s="82"/>
       <c r="F221" s="87"/>
@@ -8913,7 +8915,7 @@
         <v>36</v>
       </c>
       <c r="D222" s="123" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E222" s="82"/>
       <c r="F222" s="87"/>
@@ -8937,7 +8939,7 @@
         <v>36</v>
       </c>
       <c r="D223" s="123" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="E223" s="82"/>
       <c r="F223" s="87"/>
@@ -8961,7 +8963,7 @@
         <v>36</v>
       </c>
       <c r="D224" s="123" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="E224" s="82"/>
       <c r="F224" s="87"/>
@@ -8987,7 +8989,7 @@
         <v>36</v>
       </c>
       <c r="D225" s="123" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E225" s="82"/>
       <c r="F225" s="87"/>
@@ -9013,7 +9015,7 @@
         <v>36</v>
       </c>
       <c r="D226" s="123" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="E226" s="82"/>
       <c r="F226" s="87" t="s">
@@ -9051,7 +9053,7 @@
         <v>36</v>
       </c>
       <c r="D227" s="123" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="E227" s="82"/>
       <c r="F227" s="87"/>
@@ -9079,7 +9081,7 @@
         <v>36</v>
       </c>
       <c r="D228" s="123" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E228" s="82"/>
       <c r="F228" s="87"/>
@@ -9107,7 +9109,7 @@
         <v>301</v>
       </c>
       <c r="D229" s="123" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="E229" s="82"/>
       <c r="F229" s="87"/>
@@ -9133,7 +9135,7 @@
         <v>36</v>
       </c>
       <c r="D230" s="123" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="E230" s="82"/>
       <c r="F230" s="87"/>
@@ -9161,7 +9163,7 @@
         <v>36</v>
       </c>
       <c r="D231" s="123" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E231" s="82"/>
       <c r="F231" s="87"/>
@@ -9189,7 +9191,7 @@
         <v>36</v>
       </c>
       <c r="D232" s="123" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="E232" s="82"/>
       <c r="F232" s="87" t="s">
@@ -9219,7 +9221,7 @@
         <v>36</v>
       </c>
       <c r="D233" s="123" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E233" s="82"/>
       <c r="F233" s="87"/>
@@ -9247,7 +9249,7 @@
         <v>257</v>
       </c>
       <c r="D234" s="123" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="E234" s="82"/>
       <c r="F234" s="93" t="s">
@@ -9277,7 +9279,7 @@
         <v>36</v>
       </c>
       <c r="D235" s="123" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E235" s="82"/>
       <c r="F235" s="87"/>
@@ -9301,7 +9303,7 @@
         <v>36</v>
       </c>
       <c r="D236" s="123" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="E236" s="82"/>
       <c r="F236" s="87"/>
@@ -9325,7 +9327,7 @@
         <v>36</v>
       </c>
       <c r="D237" s="123" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E237" s="82"/>
       <c r="F237" s="87"/>
@@ -9349,7 +9351,7 @@
         <v>36</v>
       </c>
       <c r="D238" s="123" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="E238" s="82"/>
       <c r="F238" s="87"/>
@@ -9368,7 +9370,7 @@
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A239" s="154" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="B239" s="154"/>
       <c r="C239" s="154"/>
@@ -9391,13 +9393,13 @@
         <v>26</v>
       </c>
       <c r="B240" s="83" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C240" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D240" s="81" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="E240" s="82"/>
       <c r="F240" s="87"/>
@@ -9408,7 +9410,7 @@
       <c r="K240" s="83"/>
       <c r="L240" s="83"/>
       <c r="M240" s="81" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="N240" s="82"/>
       <c r="O240" s="82"/>
@@ -9416,7 +9418,7 @@
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A241" s="151" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="B241" s="152"/>
       <c r="C241" s="152"/>
@@ -9439,26 +9441,26 @@
         <v>26</v>
       </c>
       <c r="B242" s="83" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C242" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D242" s="81" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="E242" s="82"/>
       <c r="F242" s="87"/>
       <c r="G242" s="87"/>
       <c r="H242" s="94"/>
       <c r="I242" s="81" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="J242" s="83"/>
       <c r="K242" s="83"/>
       <c r="L242" s="83"/>
       <c r="M242" s="81" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="N242" s="82"/>
       <c r="O242" s="82"/>
@@ -9466,7 +9468,7 @@
     </row>
     <row r="243" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A243" s="151" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="B243" s="157"/>
       <c r="C243" s="152"/>
@@ -9493,7 +9495,7 @@
         <v>36</v>
       </c>
       <c r="D244" s="123" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="I244" s="123"/>
       <c r="J244" s="144"/>
@@ -9510,7 +9512,7 @@
         <v>36</v>
       </c>
       <c r="D245" s="123" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="I245" s="123"/>
       <c r="J245" s="144"/>
@@ -9527,7 +9529,7 @@
         <v>36</v>
       </c>
       <c r="D246" s="123" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="I246" s="123"/>
       <c r="J246" s="144"/>
@@ -9544,7 +9546,7 @@
         <v>36</v>
       </c>
       <c r="D247" s="123" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="I247" s="123"/>
       <c r="J247" s="144"/>
@@ -9561,7 +9563,7 @@
         <v>36</v>
       </c>
       <c r="D248" s="123" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="I248" s="123" t="s">
         <v>45</v>
@@ -9572,7 +9574,7 @@
       <c r="K248" s="123"/>
       <c r="L248" s="141"/>
       <c r="M248" s="123" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="249" spans="1:16" x14ac:dyDescent="0.2">
@@ -9600,13 +9602,13 @@
         <v>26</v>
       </c>
       <c r="B250" s="83" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="C250" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D250" s="81" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E250" s="82"/>
       <c r="F250" s="87"/>
@@ -9617,7 +9619,7 @@
       <c r="K250" s="83"/>
       <c r="L250" s="83"/>
       <c r="M250" s="81" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="N250" s="82"/>
       <c r="O250" s="82"/>
@@ -9648,13 +9650,13 @@
         <v>26</v>
       </c>
       <c r="B252" s="83" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C252" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D252" s="81" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E252" s="82"/>
       <c r="F252" s="87"/>
@@ -9665,7 +9667,7 @@
       <c r="K252" s="83"/>
       <c r="L252" s="83"/>
       <c r="M252" s="81" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="N252" s="82"/>
       <c r="O252" s="82"/>
@@ -9696,13 +9698,13 @@
         <v>26</v>
       </c>
       <c r="B254" s="83" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C254" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D254" s="81" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E254" s="82"/>
       <c r="F254" s="87"/>
@@ -9713,7 +9715,7 @@
       <c r="K254" s="83"/>
       <c r="L254" s="83"/>
       <c r="M254" s="81" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="N254" s="82"/>
       <c r="O254" s="82"/>
@@ -9744,13 +9746,13 @@
         <v>26</v>
       </c>
       <c r="B256" s="83" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C256" s="115" t="s">
         <v>36</v>
       </c>
       <c r="D256" s="81" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="E256" s="82"/>
       <c r="F256" s="87"/>
@@ -11345,16 +11347,16 @@
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8E7B11B-235E-4143-B901-98294EDB0157}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="65eb73cc-43b1-4677-9773-18a81d166a12"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="15fa1163-52ae-44c9-9338-260724b6ed78"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="65eb73cc-43b1-4677-9773-18a81d166a12"/>
-    <ds:schemaRef ds:uri="15fa1163-52ae-44c9-9338-260724b6ed78"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Fix validation issues with Medication.text element and updated Excel with correct path for quantity element
</commit_message>
<xml_diff>
--- a/python-maps/documentation/CDA2FHIR_elga_eMed_groups.xlsx
+++ b/python-maps/documentation/CDA2FHIR_elga_eMed_groups.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maximilian/Documents/BlackTusk/Bundesrechenzentrum/CDA2FHIR/CDA2FHIR/python-maps/documentation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{374371A5-9F37-8043-9243-064C66F7F4B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED6DAA9B-9314-1246-A286-D4E62A3350CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2505,18 +2505,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2524,22 +2516,30 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="20" fillId="17" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3593,21 +3593,21 @@
       <c r="P14" s="82"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="154" t="s">
+      <c r="A15" s="152" t="s">
         <v>441</v>
       </c>
-      <c r="B15" s="154"/>
-      <c r="C15" s="154"/>
-      <c r="D15" s="155"/>
-      <c r="E15" s="155"/>
-      <c r="F15" s="155"/>
-      <c r="G15" s="155"/>
-      <c r="H15" s="154"/>
-      <c r="I15" s="156"/>
-      <c r="J15" s="154"/>
-      <c r="K15" s="154"/>
-      <c r="L15" s="154"/>
-      <c r="M15" s="154"/>
+      <c r="B15" s="152"/>
+      <c r="C15" s="152"/>
+      <c r="D15" s="153"/>
+      <c r="E15" s="153"/>
+      <c r="F15" s="153"/>
+      <c r="G15" s="153"/>
+      <c r="H15" s="152"/>
+      <c r="I15" s="154"/>
+      <c r="J15" s="152"/>
+      <c r="K15" s="152"/>
+      <c r="L15" s="152"/>
+      <c r="M15" s="152"/>
       <c r="N15" s="82"/>
       <c r="O15" s="82"/>
       <c r="P15" s="82"/>
@@ -4223,19 +4223,19 @@
       <c r="P38" s="82"/>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A39" s="151" t="s">
+      <c r="A39" s="158" t="s">
         <v>442</v>
       </c>
-      <c r="B39" s="152"/>
-      <c r="C39" s="152"/>
-      <c r="D39" s="152"/>
-      <c r="E39" s="152"/>
-      <c r="F39" s="152"/>
-      <c r="G39" s="152"/>
-      <c r="H39" s="152"/>
-      <c r="I39" s="152"/>
-      <c r="J39" s="152"/>
-      <c r="K39" s="153"/>
+      <c r="B39" s="159"/>
+      <c r="C39" s="159"/>
+      <c r="D39" s="159"/>
+      <c r="E39" s="159"/>
+      <c r="F39" s="159"/>
+      <c r="G39" s="159"/>
+      <c r="H39" s="159"/>
+      <c r="I39" s="159"/>
+      <c r="J39" s="159"/>
+      <c r="K39" s="160"/>
       <c r="L39" s="100"/>
       <c r="M39" s="100"/>
       <c r="N39" s="82"/>
@@ -4479,19 +4479,19 @@
       <c r="P48" s="82"/>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A49" s="151" t="s">
+      <c r="A49" s="158" t="s">
         <v>201</v>
       </c>
-      <c r="B49" s="152"/>
-      <c r="C49" s="152"/>
-      <c r="D49" s="152"/>
-      <c r="E49" s="152"/>
-      <c r="F49" s="152"/>
-      <c r="G49" s="152"/>
-      <c r="H49" s="152"/>
-      <c r="I49" s="152"/>
-      <c r="J49" s="152"/>
-      <c r="K49" s="152"/>
+      <c r="B49" s="159"/>
+      <c r="C49" s="159"/>
+      <c r="D49" s="159"/>
+      <c r="E49" s="159"/>
+      <c r="F49" s="159"/>
+      <c r="G49" s="159"/>
+      <c r="H49" s="159"/>
+      <c r="I49" s="159"/>
+      <c r="J49" s="159"/>
+      <c r="K49" s="159"/>
       <c r="L49" s="101"/>
       <c r="M49" s="100"/>
       <c r="N49" s="82"/>
@@ -4681,21 +4681,21 @@
       <c r="P56" s="82"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A57" s="159" t="s">
+      <c r="A57" s="155" t="s">
         <v>202</v>
       </c>
-      <c r="B57" s="149"/>
-      <c r="C57" s="149"/>
-      <c r="D57" s="149"/>
-      <c r="E57" s="149"/>
-      <c r="F57" s="149"/>
-      <c r="G57" s="149"/>
-      <c r="H57" s="149"/>
-      <c r="I57" s="160"/>
-      <c r="J57" s="160"/>
-      <c r="K57" s="160"/>
-      <c r="L57" s="149"/>
-      <c r="M57" s="161"/>
+      <c r="B57" s="150"/>
+      <c r="C57" s="150"/>
+      <c r="D57" s="150"/>
+      <c r="E57" s="150"/>
+      <c r="F57" s="150"/>
+      <c r="G57" s="150"/>
+      <c r="H57" s="150"/>
+      <c r="I57" s="156"/>
+      <c r="J57" s="156"/>
+      <c r="K57" s="156"/>
+      <c r="L57" s="150"/>
+      <c r="M57" s="157"/>
       <c r="N57" s="82"/>
       <c r="O57" s="82"/>
       <c r="P57" s="82"/>
@@ -4788,10 +4788,10 @@
       <c r="G61" s="103"/>
       <c r="H61" s="103"/>
       <c r="I61" s="102"/>
-      <c r="J61" s="148"/>
-      <c r="K61" s="148"/>
-      <c r="L61" s="149"/>
-      <c r="M61" s="150"/>
+      <c r="J61" s="149"/>
+      <c r="K61" s="149"/>
+      <c r="L61" s="150"/>
+      <c r="M61" s="151"/>
       <c r="N61" s="82"/>
       <c r="O61" s="82"/>
       <c r="P61" s="82"/>
@@ -5237,10 +5237,10 @@
       <c r="G79" s="103"/>
       <c r="H79" s="103"/>
       <c r="I79" s="102"/>
-      <c r="J79" s="148"/>
-      <c r="K79" s="148"/>
-      <c r="L79" s="149"/>
-      <c r="M79" s="150"/>
+      <c r="J79" s="149"/>
+      <c r="K79" s="149"/>
+      <c r="L79" s="150"/>
+      <c r="M79" s="151"/>
       <c r="N79" s="82"/>
       <c r="O79" s="82"/>
       <c r="P79" s="82"/>
@@ -8776,7 +8776,7 @@
       <c r="C217" s="115" t="s">
         <v>36</v>
       </c>
-      <c r="D217" s="164" t="s">
+      <c r="D217" s="148" t="s">
         <v>432</v>
       </c>
       <c r="E217" s="82"/>
@@ -8804,7 +8804,7 @@
       <c r="C218" s="115" t="s">
         <v>257</v>
       </c>
-      <c r="D218" s="164" t="s">
+      <c r="D218" s="148" t="s">
         <v>433</v>
       </c>
       <c r="E218" s="82"/>
@@ -9369,21 +9369,21 @@
       <c r="P238" s="18"/>
     </row>
     <row r="239" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A239" s="154" t="s">
+      <c r="A239" s="152" t="s">
         <v>441</v>
       </c>
-      <c r="B239" s="154"/>
-      <c r="C239" s="154"/>
-      <c r="D239" s="155"/>
-      <c r="E239" s="155"/>
-      <c r="F239" s="155"/>
-      <c r="G239" s="155"/>
-      <c r="H239" s="154"/>
-      <c r="I239" s="156"/>
-      <c r="J239" s="154"/>
-      <c r="K239" s="154"/>
-      <c r="L239" s="154"/>
-      <c r="M239" s="154"/>
+      <c r="B239" s="152"/>
+      <c r="C239" s="152"/>
+      <c r="D239" s="153"/>
+      <c r="E239" s="153"/>
+      <c r="F239" s="153"/>
+      <c r="G239" s="153"/>
+      <c r="H239" s="152"/>
+      <c r="I239" s="154"/>
+      <c r="J239" s="152"/>
+      <c r="K239" s="152"/>
+      <c r="L239" s="152"/>
+      <c r="M239" s="152"/>
       <c r="N239" s="82"/>
       <c r="O239" s="82"/>
       <c r="P239" s="82"/>
@@ -9417,19 +9417,19 @@
       <c r="P240" s="82"/>
     </row>
     <row r="241" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A241" s="151" t="s">
+      <c r="A241" s="158" t="s">
         <v>442</v>
       </c>
-      <c r="B241" s="152"/>
-      <c r="C241" s="152"/>
-      <c r="D241" s="152"/>
-      <c r="E241" s="152"/>
-      <c r="F241" s="152"/>
-      <c r="G241" s="152"/>
-      <c r="H241" s="152"/>
-      <c r="I241" s="152"/>
-      <c r="J241" s="152"/>
-      <c r="K241" s="153"/>
+      <c r="B241" s="159"/>
+      <c r="C241" s="159"/>
+      <c r="D241" s="159"/>
+      <c r="E241" s="159"/>
+      <c r="F241" s="159"/>
+      <c r="G241" s="159"/>
+      <c r="H241" s="159"/>
+      <c r="I241" s="159"/>
+      <c r="J241" s="159"/>
+      <c r="K241" s="160"/>
       <c r="L241" s="100"/>
       <c r="M241" s="100"/>
       <c r="N241" s="82"/>
@@ -9467,19 +9467,19 @@
       <c r="P242" s="82"/>
     </row>
     <row r="243" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A243" s="151" t="s">
+      <c r="A243" s="158" t="s">
         <v>448</v>
       </c>
-      <c r="B243" s="157"/>
-      <c r="C243" s="152"/>
-      <c r="D243" s="152"/>
-      <c r="E243" s="152"/>
-      <c r="F243" s="152"/>
-      <c r="G243" s="152"/>
-      <c r="H243" s="152"/>
-      <c r="I243" s="157"/>
-      <c r="J243" s="157"/>
-      <c r="K243" s="158"/>
+      <c r="B243" s="161"/>
+      <c r="C243" s="159"/>
+      <c r="D243" s="159"/>
+      <c r="E243" s="159"/>
+      <c r="F243" s="159"/>
+      <c r="G243" s="159"/>
+      <c r="H243" s="159"/>
+      <c r="I243" s="161"/>
+      <c r="J243" s="161"/>
+      <c r="K243" s="162"/>
       <c r="L243" s="140"/>
       <c r="M243" s="140"/>
       <c r="N243" s="82"/>
@@ -9589,10 +9589,10 @@
       <c r="G249" s="103"/>
       <c r="H249" s="103"/>
       <c r="I249" s="102"/>
-      <c r="J249" s="148"/>
-      <c r="K249" s="148"/>
-      <c r="L249" s="149"/>
-      <c r="M249" s="150"/>
+      <c r="J249" s="149"/>
+      <c r="K249" s="149"/>
+      <c r="L249" s="150"/>
+      <c r="M249" s="151"/>
       <c r="N249" s="82"/>
       <c r="O249" s="82"/>
       <c r="P249" s="82"/>
@@ -9637,10 +9637,10 @@
       <c r="G251" s="103"/>
       <c r="H251" s="103"/>
       <c r="I251" s="102"/>
-      <c r="J251" s="148"/>
-      <c r="K251" s="148"/>
-      <c r="L251" s="149"/>
-      <c r="M251" s="150"/>
+      <c r="J251" s="149"/>
+      <c r="K251" s="149"/>
+      <c r="L251" s="150"/>
+      <c r="M251" s="151"/>
       <c r="N251" s="82"/>
       <c r="O251" s="82"/>
       <c r="P251" s="82"/>
@@ -9771,17 +9771,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="J251:M251"/>
+    <mergeCell ref="A241:K241"/>
+    <mergeCell ref="A239:M239"/>
+    <mergeCell ref="A243:K243"/>
+    <mergeCell ref="J249:M249"/>
     <mergeCell ref="J79:M79"/>
     <mergeCell ref="A15:M15"/>
     <mergeCell ref="A57:M57"/>
     <mergeCell ref="J61:M61"/>
     <mergeCell ref="A39:K39"/>
     <mergeCell ref="A49:K49"/>
-    <mergeCell ref="J251:M251"/>
-    <mergeCell ref="A241:K241"/>
-    <mergeCell ref="A239:M239"/>
-    <mergeCell ref="A243:K243"/>
-    <mergeCell ref="J249:M249"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A56 A58:A60 A62:A78 A80:A96 A98:A151 A153:A158 A181:A193 A195:A248 A250 A252 A254 A256:A1048576">
     <cfRule type="cellIs" dxfId="10" priority="17" operator="equal">
@@ -9840,12 +9840,12 @@
     <row r="1" spans="1:26" ht="20" x14ac:dyDescent="0.2">
       <c r="A1" s="26"/>
       <c r="B1" s="27"/>
-      <c r="C1" s="162" t="s">
+      <c r="C1" s="163" t="s">
         <v>105</v>
       </c>
-      <c r="D1" s="162"/>
-      <c r="E1" s="163"/>
-      <c r="F1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="164"/>
+      <c r="F1" s="164"/>
       <c r="I1" s="26"/>
       <c r="J1" s="28"/>
       <c r="K1" s="28"/>
@@ -11102,14 +11102,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="15fa1163-52ae-44c9-9338-260724b6ed78" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65eb73cc-43b1-4677-9773-18a81d166a12">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11336,27 +11334,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="15fa1163-52ae-44c9-9338-260724b6ed78" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65eb73cc-43b1-4677-9773-18a81d166a12">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8E7B11B-235E-4143-B901-98294EDB0157}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E01F75D2-18D7-4457-A217-CD23D85DC8FD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="65eb73cc-43b1-4677-9773-18a81d166a12"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="15fa1163-52ae-44c9-9338-260724b6ed78"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11381,9 +11372,18 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E01F75D2-18D7-4457-A217-CD23D85DC8FD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A8E7B11B-235E-4143-B901-98294EDB0157}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="65eb73cc-43b1-4677-9773-18a81d166a12"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="15fa1163-52ae-44c9-9338-260724b6ed78"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>